<commit_message>
Met à jour le corpus Mosar et les contrôles statistiques
</commit_message>
<xml_diff>
--- a/data/Recensement-revues-stat.xlsx
+++ b/data/Recensement-revues-stat.xlsx
@@ -2369,26 +2369,6 @@
           <t>Archéologie</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>numérique</t>
@@ -2412,11 +2392,6 @@
       <c r="R18" t="inlineStr">
         <is>
           <t>Pépinière</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>?</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">

</xml_diff>